<commit_message>
Code review: find the next "&" once, and test a format that it fixes
Changes from the code review of this PR:

- Checking every attribute value for "&" made SaxParser slower over a
  whole sheet, which SheetBoundsHandler scans without a dimension. Keep
  the position of the next "&", as the parser does for its other
  delimiters, and look for it again only once past it.
- The fixture now has the number 5 in the format 0 "R&D & Co", which was
  read as a date in 1900, since the letters of each &amp; counted as
  month codes. Test that it is read as 5, a fix that this PR makes on
  its own, and that the attributes are unescaped at every chunk size.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/files/sheet-name-entities.xlsx
+++ b/test/files/sheet-name-entities.xlsx
@@ -17,7 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0 &quot;R&amp;D &amp; Co&quot;"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -47,8 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -414,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -422,6 +425,9 @@
         <is>
           <t>first</t>
         </is>
+      </c>
+      <c r="B1" s="1" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>